<commit_message>
Added label maps to export excel report
</commit_message>
<xml_diff>
--- a/template/chiffrage_template.xlsx
+++ b/template/chiffrage_template.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adonfut\Desktop\Code\HET_3\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4645AF-B686-455A-81A0-0E842F96496C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDEDB55-9150-4F17-9428-5E8399575A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="2415" windowWidth="21840" windowHeight="13140" xr2:uid="{4885B836-D54B-4C79-99DC-EA9E6211BFFA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4885B836-D54B-4C79-99DC-EA9E6211BFFA}"/>
   </bookViews>
   <sheets>
     <sheet name="chiffrage" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">chiffrage!$B$1:$F$41</definedName>
   </definedNames>
@@ -861,119 +858,14 @@
     <xf numFmtId="1" fontId="0" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="5" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1042,14 +934,6 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1090,6 +974,119 @@
     </xf>
     <xf numFmtId="1" fontId="8" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1173,92 +1170,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="chiffrage"/>
-      <sheetName val="prepa ORTEMS"/>
-      <sheetName val="quest LABO"/>
-      <sheetName val="définition"/>
-      <sheetName val="abandonné"/>
-      <sheetName val="liste valeurs"/>
-      <sheetName val="data produit"/>
-      <sheetName val="data produit marine mil"/>
-      <sheetName val="data options"/>
-      <sheetName val="tri calculs"/>
-      <sheetName val=" data marine new"/>
-      <sheetName val="data calculs marine old"/>
-      <sheetName val="data LPDC marine"/>
-      <sheetName val="data options marine"/>
-      <sheetName val="tri mach mil"/>
-      <sheetName val="quest calculs"/>
-      <sheetName val="Calculs pris"/>
-      <sheetName val="quest options"/>
-      <sheetName val="Options prises"/>
-      <sheetName val="data LPDC"/>
-      <sheetName val="quest LPDC"/>
-      <sheetName val="tri1 LPDC"/>
-      <sheetName val="tri options"/>
-      <sheetName val="data calculs"/>
-      <sheetName val="LPDC prise"/>
-      <sheetName val="révision"/>
-      <sheetName val="info gen"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5">
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>asynchrone à bagues</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21" t="str">
-            <v xml:space="preserve">marine militaire </v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>jeu de bagues Asynch</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1547,132 +1458,132 @@
       <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:74" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="41"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="79"/>
     </row>
     <row r="3" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="29" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="18"/>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="82"/>
     </row>
     <row r="4" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="25" t="s">
         <v>15</v>
       </c>
       <c r="C4" s="12"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="47"/>
+      <c r="D4" s="83"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="85"/>
     </row>
     <row r="5" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
         <v>17</v>
       </c>
       <c r="C5" s="13"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="47"/>
+      <c r="D5" s="83"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="85"/>
     </row>
     <row r="6" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="26" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="14"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="47"/>
+      <c r="D6" s="83"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="85"/>
     </row>
     <row r="7" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="26" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="13"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="47"/>
+      <c r="D7" s="83"/>
+      <c r="E7" s="84"/>
+      <c r="F7" s="85"/>
     </row>
     <row r="8" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="26" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="13"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="46"/>
-      <c r="F8" s="47"/>
+      <c r="D8" s="83"/>
+      <c r="E8" s="84"/>
+      <c r="F8" s="85"/>
     </row>
     <row r="9" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="26" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="13"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="47"/>
+      <c r="D9" s="83"/>
+      <c r="E9" s="84"/>
+      <c r="F9" s="85"/>
     </row>
     <row r="10" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="26" t="s">
         <v>21</v>
       </c>
       <c r="C10" s="13"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="47"/>
+      <c r="D10" s="83"/>
+      <c r="E10" s="84"/>
+      <c r="F10" s="85"/>
     </row>
     <row r="11" spans="1:74" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="26" t="s">
         <v>22</v>
       </c>
       <c r="C11" s="13"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="47"/>
+      <c r="D11" s="83"/>
+      <c r="E11" s="84"/>
+      <c r="F11" s="85"/>
     </row>
     <row r="12" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="26" t="s">
         <v>23</v>
       </c>
       <c r="C12" s="23"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="46"/>
-      <c r="F12" s="47"/>
+      <c r="D12" s="83"/>
+      <c r="E12" s="84"/>
+      <c r="F12" s="85"/>
     </row>
     <row r="13" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="26" t="s">
         <v>24</v>
       </c>
       <c r="C13" s="13"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="46"/>
-      <c r="F13" s="47"/>
+      <c r="D13" s="83"/>
+      <c r="E13" s="84"/>
+      <c r="F13" s="85"/>
     </row>
     <row r="14" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="27" t="s">
         <v>26</v>
       </c>
       <c r="C14" s="13"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="47"/>
+      <c r="D14" s="83"/>
+      <c r="E14" s="84"/>
+      <c r="F14" s="85"/>
     </row>
     <row r="15" spans="1:74" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="28" t="s">
         <v>27</v>
       </c>
       <c r="C15" s="19"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="50"/>
+      <c r="D15" s="86"/>
+      <c r="E15" s="87"/>
+      <c r="F15" s="88"/>
     </row>
     <row r="16" spans="1:74" s="5" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4"/>
@@ -1758,15 +1669,15 @@
     </row>
     <row r="17" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="97" t="s">
+      <c r="C17" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="98"/>
-      <c r="E17" s="98"/>
-      <c r="F17" s="99"/>
+      <c r="D17" s="64"/>
+      <c r="E17" s="64"/>
+      <c r="F17" s="65"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -1838,13 +1749,13 @@
     </row>
     <row r="18" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
-      <c r="B18" s="54"/>
-      <c r="C18" s="72" t="s">
+      <c r="B18" s="94"/>
+      <c r="C18" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="73"/>
-      <c r="E18" s="73"/>
-      <c r="F18" s="100"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="66"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -1912,13 +1823,13 @@
     </row>
     <row r="19" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
-      <c r="B19" s="54"/>
-      <c r="C19" s="72" t="s">
+      <c r="B19" s="94"/>
+      <c r="C19" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="73"/>
-      <c r="E19" s="73"/>
-      <c r="F19" s="100"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="66"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -1986,13 +1897,13 @@
     </row>
     <row r="20" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
-      <c r="B20" s="55"/>
-      <c r="C20" s="72" t="s">
+      <c r="B20" s="95"/>
+      <c r="C20" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="73"/>
-      <c r="E20" s="73"/>
-      <c r="F20" s="100"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="66"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -2060,13 +1971,13 @@
     </row>
     <row r="21" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
-      <c r="B21" s="56" t="s">
+      <c r="B21" s="96" t="s">
         <v>2</v>
       </c>
-      <c r="C21" s="74"/>
-      <c r="D21" s="75"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="101"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="67"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -2134,11 +2045,11 @@
     </row>
     <row r="22" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
-      <c r="B22" s="57"/>
-      <c r="C22" s="74"/>
-      <c r="D22" s="75"/>
-      <c r="E22" s="76"/>
-      <c r="F22" s="101"/>
+      <c r="B22" s="97"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="67"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -2206,11 +2117,11 @@
     </row>
     <row r="23" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
-      <c r="B23" s="57"/>
-      <c r="C23" s="74"/>
-      <c r="D23" s="75"/>
-      <c r="E23" s="76"/>
-      <c r="F23" s="101"/>
+      <c r="B23" s="97"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="67"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -2278,11 +2189,11 @@
     </row>
     <row r="24" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="57"/>
-      <c r="C24" s="74"/>
-      <c r="D24" s="75"/>
-      <c r="E24" s="76"/>
-      <c r="F24" s="101"/>
+      <c r="B24" s="97"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="67"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
@@ -2350,11 +2261,11 @@
     </row>
     <row r="25" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
-      <c r="B25" s="58"/>
-      <c r="C25" s="74"/>
-      <c r="D25" s="75"/>
-      <c r="E25" s="76"/>
-      <c r="F25" s="101"/>
+      <c r="B25" s="98"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="67"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
@@ -2422,12 +2333,12 @@
     </row>
     <row r="26" spans="1:74" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
-      <c r="B26" s="59" t="s">
+      <c r="B26" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="C26" s="77"/>
-      <c r="D26" s="78"/>
-      <c r="E26" s="79"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="47"/>
       <c r="F26" s="33"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -2496,15 +2407,12 @@
     </row>
     <row r="27" spans="1:74" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
-      <c r="B27" s="60" t="s">
+      <c r="B27" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="C27" s="80" t="str">
-        <f>IF($C$9&lt;&gt;'[1]liste valeurs'!$A$21,IF(C8='[1]liste valeurs'!A8,'[1]tri options'!A2,""),"")</f>
-        <v/>
-      </c>
-      <c r="D27" s="81"/>
-      <c r="E27" s="82"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="50"/>
       <c r="F27" s="34"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -2572,128 +2480,128 @@
       <c r="BR27" s="4"/>
     </row>
     <row r="28" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B28" s="61" t="s">
+      <c r="B28" s="104" t="s">
         <v>5</v>
       </c>
-      <c r="C28" s="83" t="s">
+      <c r="C28" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="D28" s="84"/>
-      <c r="E28" s="85"/>
-      <c r="F28" s="102"/>
+      <c r="D28" s="52"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="68"/>
     </row>
     <row r="29" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B29" s="62"/>
-      <c r="C29" s="83" t="s">
+      <c r="B29" s="105"/>
+      <c r="C29" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="D29" s="84"/>
-      <c r="E29" s="85"/>
-      <c r="F29" s="102"/>
+      <c r="D29" s="52"/>
+      <c r="E29" s="53"/>
+      <c r="F29" s="68"/>
     </row>
     <row r="30" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B30" s="63" t="s">
+      <c r="B30" s="102" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="86" t="s">
+      <c r="C30" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="D30" s="87"/>
-      <c r="E30" s="88"/>
-      <c r="F30" s="103"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="69"/>
     </row>
     <row r="31" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B31" s="64"/>
-      <c r="C31" s="86" t="s">
+      <c r="B31" s="103"/>
+      <c r="C31" s="54" t="s">
         <v>34</v>
       </c>
-      <c r="D31" s="87"/>
-      <c r="E31" s="88"/>
-      <c r="F31" s="103"/>
+      <c r="D31" s="55"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="69"/>
     </row>
     <row r="32" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B32" s="65" t="s">
+      <c r="B32" s="99" t="s">
         <v>12</v>
       </c>
-      <c r="C32" s="89" t="s">
+      <c r="C32" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="D32" s="90"/>
-      <c r="E32" s="91"/>
-      <c r="F32" s="104"/>
+      <c r="D32" s="58"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="70"/>
     </row>
     <row r="33" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B33" s="66"/>
-      <c r="C33" s="89" t="s">
+      <c r="B33" s="100"/>
+      <c r="C33" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="D33" s="90"/>
-      <c r="E33" s="91"/>
-      <c r="F33" s="104"/>
+      <c r="D33" s="58"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="70"/>
     </row>
     <row r="34" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B34" s="66"/>
-      <c r="C34" s="89" t="s">
+      <c r="B34" s="100"/>
+      <c r="C34" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="D34" s="90"/>
-      <c r="E34" s="91"/>
-      <c r="F34" s="104"/>
+      <c r="D34" s="58"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="70"/>
     </row>
     <row r="35" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B35" s="66"/>
-      <c r="C35" s="89" t="s">
+      <c r="B35" s="100"/>
+      <c r="C35" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="D35" s="90"/>
-      <c r="E35" s="91"/>
-      <c r="F35" s="104"/>
+      <c r="D35" s="58"/>
+      <c r="E35" s="59"/>
+      <c r="F35" s="70"/>
     </row>
     <row r="36" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B36" s="66"/>
-      <c r="C36" s="89" t="s">
+      <c r="B36" s="100"/>
+      <c r="C36" s="57" t="s">
         <v>39</v>
       </c>
-      <c r="D36" s="90"/>
-      <c r="E36" s="91"/>
-      <c r="F36" s="104"/>
+      <c r="D36" s="58"/>
+      <c r="E36" s="59"/>
+      <c r="F36" s="70"/>
     </row>
     <row r="37" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B37" s="67"/>
-      <c r="C37" s="89" t="s">
+      <c r="B37" s="101"/>
+      <c r="C37" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="D37" s="90"/>
-      <c r="E37" s="91"/>
-      <c r="F37" s="104"/>
+      <c r="D37" s="58"/>
+      <c r="E37" s="59"/>
+      <c r="F37" s="70"/>
     </row>
     <row r="38" spans="1:70" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="68" t="s">
+      <c r="B38" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="C38" s="105" t="s">
+      <c r="C38" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="D38" s="106"/>
-      <c r="E38" s="107"/>
+      <c r="D38" s="72"/>
+      <c r="E38" s="73"/>
       <c r="F38" s="35"/>
     </row>
     <row r="39" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B39" s="92" t="s">
+      <c r="B39" s="106" t="s">
         <v>8</v>
       </c>
-      <c r="C39" s="93"/>
-      <c r="D39" s="94"/>
-      <c r="E39" s="95"/>
-      <c r="F39" s="96"/>
+      <c r="C39" s="107"/>
+      <c r="D39" s="60"/>
+      <c r="E39" s="61"/>
+      <c r="F39" s="62"/>
     </row>
     <row r="40" spans="1:70" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="69" t="s">
+      <c r="B40" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="C40" s="70"/>
+      <c r="C40" s="92"/>
       <c r="D40" s="15"/>
-      <c r="E40" s="71"/>
+      <c r="E40" s="39"/>
       <c r="F40" s="16"/>
     </row>
     <row r="41" spans="1:70" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -2701,18 +2609,18 @@
         <v>43</v>
       </c>
       <c r="C41" s="30"/>
-      <c r="D41" s="51" t="s">
+      <c r="D41" s="89" t="s">
         <v>44</v>
       </c>
-      <c r="E41" s="52"/>
+      <c r="E41" s="90"/>
       <c r="F41" s="31"/>
     </row>
     <row r="42" spans="1:70" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="36"/>
-      <c r="C42" s="37"/>
-      <c r="D42" s="37"/>
-      <c r="E42" s="37"/>
-      <c r="F42" s="38"/>
+      <c r="B42" s="74"/>
+      <c r="C42" s="75"/>
+      <c r="D42" s="75"/>
+      <c r="E42" s="75"/>
+      <c r="F42" s="76"/>
     </row>
     <row r="44" spans="1:70" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>

</xml_diff>

<commit_message>
v1.2.0 Séparation de NRC et RC
</commit_message>
<xml_diff>
--- a/template/chiffrage_template.xlsx
+++ b/template/chiffrage_template.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adonfut\Desktop\Code\HET_3\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F683940-773B-431B-9657-2C16F64FDEAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD926AAF-EB8A-412A-8C1F-60FBC16DEBF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4885B836-D54B-4C79-99DC-EA9E6211BFFA}"/>
+    <workbookView xWindow="28680" yWindow="2415" windowWidth="21840" windowHeight="13140" xr2:uid="{4885B836-D54B-4C79-99DC-EA9E6211BFFA}"/>
   </bookViews>
   <sheets>
     <sheet name="chiffrage" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">chiffrage!$B$1:$F$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">chiffrage!$B$1:$F$33</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="51">
   <si>
     <t>Chiffrage des heures études</t>
   </si>
@@ -59,15 +59,6 @@
     <t>LABO</t>
   </si>
   <si>
-    <t>DIVERS</t>
-  </si>
-  <si>
-    <t>Machine N°1</t>
-  </si>
-  <si>
-    <t>TOTAL pour N machines</t>
-  </si>
-  <si>
     <t>Correction manuelle</t>
   </si>
   <si>
@@ -183,6 +174,24 @@
   </si>
   <si>
     <t>Revue de conception (ensemble)</t>
+  </si>
+  <si>
+    <t>TOTAL NRC</t>
+  </si>
+  <si>
+    <t>TOTAL RC</t>
+  </si>
+  <si>
+    <t>RC POUR N machines</t>
+  </si>
+  <si>
+    <t>DIVERS RC</t>
+  </si>
+  <si>
+    <t>DIVERS NRC</t>
+  </si>
+  <si>
+    <t>TOTAL RC + NRC</t>
   </si>
 </sst>
 </file>
@@ -192,16 +201,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yy;@"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -268,14 +269,29 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="14"/>
+      <color theme="4" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="4" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -337,7 +353,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -696,19 +712,71 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
@@ -718,13 +786,6 @@
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -733,288 +794,296 @@
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="9" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="8" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="8" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="9" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="8" fillId="9" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="4" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="8" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="9" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="7" fillId="9" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="9" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="9" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="7" fillId="9" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="9" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="9" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="9" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="9" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="9" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="8" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="6" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="7" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="9" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="5" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="5" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1366,15 +1435,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" style="4"/>
     <col min="2" max="2" width="36.140625" style="5" customWidth="1"/>
     <col min="3" max="3" width="40" style="4" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="8" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" style="8" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" style="6" customWidth="1"/>
     <col min="7" max="16384" width="10.85546875" style="4"/>
   </cols>
   <sheetData>
@@ -1386,430 +1455,434 @@
       <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:6" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="81" t="s">
+      <c r="B2" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="84"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="11"/>
+      <c r="D3" s="85" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" s="86"/>
+      <c r="F3" s="87"/>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B4" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="88"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="90"/>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="84" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="85"/>
-      <c r="F3" s="86"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="C5" s="9"/>
+      <c r="D5" s="88"/>
+      <c r="E5" s="89"/>
+      <c r="F5" s="90"/>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B6" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="10"/>
+      <c r="D6" s="88"/>
+      <c r="E6" s="89"/>
+      <c r="F6" s="90"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="87"/>
-      <c r="E4" s="88"/>
-      <c r="F4" s="89"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="17" t="s">
+      <c r="C7" s="9"/>
+      <c r="D7" s="88"/>
+      <c r="E7" s="89"/>
+      <c r="F7" s="90"/>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B8" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="89"/>
+      <c r="F8" s="90"/>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B9" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="87"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="89"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="12"/>
-      <c r="D6" s="87"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="89"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="17" t="s">
+      <c r="C9" s="9"/>
+      <c r="D9" s="88"/>
+      <c r="E9" s="89"/>
+      <c r="F9" s="90"/>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B10" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="87"/>
-      <c r="E7" s="88"/>
-      <c r="F7" s="89"/>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="17" t="s">
+      <c r="C10" s="9"/>
+      <c r="D10" s="88"/>
+      <c r="E10" s="89"/>
+      <c r="F10" s="90"/>
+    </row>
+    <row r="11" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="87"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="89"/>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="17" t="s">
+      <c r="C11" s="9"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="89"/>
+      <c r="F11" s="90"/>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B12" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="87"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="89"/>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="17" t="s">
+      <c r="C12" s="13"/>
+      <c r="D12" s="88"/>
+      <c r="E12" s="89"/>
+      <c r="F12" s="90"/>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="87"/>
-      <c r="E10" s="88"/>
-      <c r="F10" s="89"/>
-    </row>
-    <row r="11" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="87"/>
-      <c r="E11" s="88"/>
-      <c r="F11" s="89"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B12" s="17" t="s">
+      <c r="C13" s="9"/>
+      <c r="D13" s="88"/>
+      <c r="E13" s="89"/>
+      <c r="F13" s="90"/>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B14" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="87"/>
-      <c r="E12" s="88"/>
-      <c r="F12" s="89"/>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="17" t="s">
+      <c r="C14" s="9"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="89"/>
+      <c r="F14" s="90"/>
+    </row>
+    <row r="15" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="87"/>
-      <c r="E13" s="88"/>
-      <c r="F13" s="89"/>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="87"/>
-      <c r="E14" s="88"/>
-      <c r="F14" s="89"/>
-    </row>
-    <row r="15" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="90"/>
-      <c r="E15" s="91"/>
-      <c r="F15" s="92"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="91"/>
+      <c r="E15" s="92"/>
+      <c r="F15" s="93"/>
     </row>
     <row r="16" spans="1:6" s="5" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4"/>
-      <c r="B16" s="58"/>
-      <c r="C16" s="59"/>
-      <c r="D16" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="61" t="s">
-        <v>9</v>
-      </c>
-      <c r="F16" s="62" t="s">
-        <v>10</v>
+      <c r="B16" s="27"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
-      <c r="B17" s="93" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="68" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69"/>
-      <c r="F17" s="70"/>
+      <c r="B17" s="94" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="50"/>
     </row>
     <row r="18" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
-      <c r="B18" s="94"/>
-      <c r="C18" s="71" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="72"/>
-      <c r="E18" s="72"/>
-      <c r="F18" s="73"/>
+      <c r="B18" s="95"/>
+      <c r="C18" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="52"/>
     </row>
     <row r="19" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
-      <c r="B19" s="94"/>
-      <c r="C19" s="71" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="72"/>
-      <c r="E19" s="72"/>
-      <c r="F19" s="73"/>
+      <c r="B19" s="95"/>
+      <c r="C19" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="51"/>
+      <c r="E19" s="51"/>
+      <c r="F19" s="52"/>
     </row>
     <row r="20" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
-      <c r="B20" s="95"/>
-      <c r="C20" s="71" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="72"/>
-      <c r="E20" s="72"/>
-      <c r="F20" s="73"/>
+      <c r="B20" s="96"/>
+      <c r="C20" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="51"/>
+      <c r="E20" s="51"/>
+      <c r="F20" s="52"/>
     </row>
     <row r="21" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
-      <c r="B21" s="96" t="s">
+      <c r="B21" s="97" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="28" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" s="29"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="31"/>
+      <c r="C21" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" s="53"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="55"/>
     </row>
     <row r="22" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
-      <c r="B22" s="97"/>
-      <c r="C22" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" s="29"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="31"/>
+      <c r="B22" s="98"/>
+      <c r="C22" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="53"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="55"/>
     </row>
     <row r="23" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
-      <c r="B23" s="97"/>
-      <c r="C23" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" s="29"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="31"/>
+      <c r="B23" s="98"/>
+      <c r="C23" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="53"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="55"/>
     </row>
     <row r="24" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="97"/>
-      <c r="C24" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" s="29"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="31"/>
+      <c r="B24" s="98"/>
+      <c r="C24" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="53"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="55"/>
     </row>
     <row r="25" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
-      <c r="B25" s="98"/>
-      <c r="C25" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="D25" s="29"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="31"/>
+      <c r="B25" s="99"/>
+      <c r="C25" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="53"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="55"/>
     </row>
     <row r="26" spans="1:6" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
-      <c r="B26" s="63" t="s">
+      <c r="B26" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="C26" s="64"/>
-      <c r="D26" s="65"/>
-      <c r="E26" s="66"/>
-      <c r="F26" s="67"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="56"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="58"/>
     </row>
     <row r="27" spans="1:6" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="34"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="59"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="61"/>
     </row>
     <row r="28" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B28" s="79" t="s">
+      <c r="B28" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="C28" s="35" t="s">
+      <c r="C28" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="62"/>
+      <c r="E28" s="63"/>
+      <c r="F28" s="64"/>
+    </row>
+    <row r="29" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B29" s="41"/>
+      <c r="C29" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="62"/>
+      <c r="E29" s="63"/>
+      <c r="F29" s="64"/>
+    </row>
+    <row r="30" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B30" s="39" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" s="65"/>
+      <c r="E30" s="66"/>
+      <c r="F30" s="67"/>
+    </row>
+    <row r="31" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B31" s="43"/>
+      <c r="C31" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="D31" s="68"/>
+      <c r="E31" s="69"/>
+      <c r="F31" s="70"/>
+    </row>
+    <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32" s="71"/>
+      <c r="E32" s="72"/>
+      <c r="F32" s="73"/>
+    </row>
+    <row r="33" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" s="46"/>
+      <c r="D33" s="80"/>
+      <c r="E33" s="79"/>
+      <c r="F33" s="81"/>
+    </row>
+    <row r="34" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B34" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="D28" s="36"/>
-      <c r="E28" s="37"/>
-      <c r="F28" s="38"/>
-    </row>
-    <row r="29" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B29" s="80"/>
-      <c r="C29" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="36"/>
-      <c r="E29" s="37"/>
-      <c r="F29" s="38"/>
-    </row>
-    <row r="30" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B30" s="77" t="s">
-        <v>5</v>
-      </c>
-      <c r="C30" s="39" t="s">
+      <c r="D34" s="74"/>
+      <c r="E34" s="75"/>
+      <c r="F34" s="76"/>
+    </row>
+    <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B35" s="37"/>
+      <c r="C35" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="40"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="42"/>
-    </row>
-    <row r="31" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B31" s="78"/>
-      <c r="C31" s="39" t="s">
+      <c r="D35" s="74"/>
+      <c r="E35" s="75"/>
+      <c r="F35" s="76"/>
+    </row>
+    <row r="36" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B36" s="37"/>
+      <c r="C36" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D31" s="40"/>
-      <c r="E31" s="41"/>
-      <c r="F31" s="42"/>
-    </row>
-    <row r="32" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B32" s="74" t="s">
-        <v>11</v>
-      </c>
-      <c r="C32" s="43" t="s">
+      <c r="D36" s="74"/>
+      <c r="E36" s="75"/>
+      <c r="F36" s="76"/>
+    </row>
+    <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B37" s="37"/>
+      <c r="C37" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="D32" s="44"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="46"/>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B33" s="75"/>
-      <c r="C33" s="43" t="s">
+      <c r="D37" s="74"/>
+      <c r="E37" s="75"/>
+      <c r="F37" s="76"/>
+    </row>
+    <row r="38" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B38" s="37"/>
+      <c r="C38" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="D33" s="44"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="46"/>
-    </row>
-    <row r="34" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B34" s="75"/>
-      <c r="C34" s="43" t="s">
+      <c r="D38" s="74"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="76"/>
+    </row>
+    <row r="39" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B39" s="38"/>
+      <c r="C39" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D34" s="44"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="46"/>
-    </row>
-    <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B35" s="75"/>
-      <c r="C35" s="43" t="s">
+      <c r="D39" s="74"/>
+      <c r="E39" s="75"/>
+      <c r="F39" s="76"/>
+    </row>
+    <row r="40" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C40" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="D35" s="44"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="46"/>
-    </row>
-    <row r="36" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B36" s="75"/>
-      <c r="C36" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="D36" s="44"/>
-      <c r="E36" s="45"/>
-      <c r="F36" s="46"/>
-    </row>
-    <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B37" s="76"/>
-      <c r="C37" s="43" t="s">
-        <v>38</v>
-      </c>
-      <c r="D37" s="44"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="46"/>
-    </row>
-    <row r="38" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="D38" s="47"/>
-      <c r="E38" s="48"/>
-      <c r="F38" s="49"/>
-    </row>
-    <row r="39" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B39" s="55" t="s">
-        <v>7</v>
-      </c>
-      <c r="C39" s="56"/>
-      <c r="D39" s="50"/>
-      <c r="E39" s="51"/>
-      <c r="F39" s="52"/>
-    </row>
-    <row r="40" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="54" t="s">
-        <v>8</v>
-      </c>
-      <c r="C40" s="57"/>
-      <c r="D40" s="53"/>
-      <c r="E40" s="100"/>
-      <c r="F40" s="99"/>
-    </row>
-    <row r="41" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B41" s="23"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="24"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-    </row>
-    <row r="44" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="4"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-    </row>
-    <row r="48" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="4"/>
-      <c r="B48" s="5"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-    </row>
-    <row r="49" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="4"/>
-      <c r="B49" s="5"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
-    </row>
-    <row r="50" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="4"/>
-      <c r="B50" s="5"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="9"/>
+      <c r="D40" s="71"/>
+      <c r="E40" s="72"/>
+      <c r="F40" s="73"/>
+    </row>
+    <row r="41" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="45" t="s">
+        <v>46</v>
+      </c>
+      <c r="C41" s="46"/>
+      <c r="D41" s="80"/>
+      <c r="E41" s="79"/>
+      <c r="F41" s="81"/>
+    </row>
+    <row r="42" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="45" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="46"/>
+      <c r="D42" s="80"/>
+      <c r="E42" s="79"/>
+      <c r="F42" s="81"/>
+    </row>
+    <row r="43" spans="1:6" s="1" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="4"/>
+      <c r="B43" s="47" t="s">
+        <v>50</v>
+      </c>
+      <c r="C43" s="48"/>
+      <c r="D43" s="77"/>
+      <c r="E43" s="78"/>
+      <c r="F43" s="42"/>
+    </row>
+    <row r="45" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="4"/>
+    </row>
+    <row r="46" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="4"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6"/>
+      <c r="F46" s="6"/>
+    </row>
+    <row r="47" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="4"/>
+      <c r="B47" s="5"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>